<commit_message>
style(sheets): 민요 새 타령-2 악보 행 높이 줄여 A4 맞춤 (배율 24% → 46%) + PDF 갱신
</commit_message>
<xml_diff>
--- a/sheets/민요/검수/새 타령-2.xlsx
+++ b/sheets/민요/검수/새 타령-2.xlsx
@@ -4556,7 +4556,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="6.0" customHeight="true"/>
-    <row r="2" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="166.67" customHeight="true">
+    <row r="2" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="86.96" customHeight="true">
       <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
@@ -4580,7 +4580,7 @@
       <c r="T2" s="18"/>
       <c r="U2" s="18"/>
     </row>
-    <row r="3" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="3" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B3" s="19" t="s">
         <v>77</v>
       </c>
@@ -4640,7 +4640,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="4" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B4" s="19" t="s">
         <v>77</v>
       </c>
@@ -4696,7 +4696,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="5" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B5" s="19" t="s">
         <v>77</v>
       </c>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="U5" s="22"/>
     </row>
-    <row r="6" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="6" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B6" s="19" t="s">
         <v>78</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="7" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="7" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B7" s="19" t="s">
         <v>107</v>
       </c>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="U7" s="21"/>
     </row>
-    <row r="8" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="8" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B8" s="19" t="s">
         <v>77</v>
       </c>
@@ -4892,7 +4892,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="9" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B9" s="19" t="s">
         <v>82</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="10" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B10" s="19" t="s">
         <v>84</v>
       </c>
@@ -4996,7 +4996,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="11" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B11" s="19" t="s">
         <v>55</v>
       </c>
@@ -5038,7 +5038,7 @@
       </c>
       <c r="U11" s="22"/>
     </row>
-    <row r="12" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="12" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B12" s="19" t="s">
         <v>77</v>
       </c>
@@ -5092,7 +5092,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="13" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B13" s="19" t="s">
         <v>47</v>
       </c>
@@ -5140,7 +5140,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B14" s="19" t="s">
         <v>58</v>
       </c>
@@ -5187,7 +5187,7 @@
       <c r="U14" s="22"/>
     </row>
     <row r="15" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="6.0" customHeight="true"/>
-    <row r="16" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="166.67" customHeight="true">
+    <row r="16" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="86.96" customHeight="true">
       <c r="B16" s="18" t="s">
         <v>0</v>
       </c>
@@ -5211,7 +5211,7 @@
       <c r="T16" s="18"/>
       <c r="U16" s="18"/>
     </row>
-    <row r="17" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="17" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B17" s="19"/>
       <c r="C17" s="20"/>
       <c r="D17" s="19"/>
@@ -5237,7 +5237,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="18" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="18" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B18" s="19"/>
       <c r="C18" s="21"/>
       <c r="D18" s="19"/>
@@ -5263,7 +5263,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B19" s="19"/>
       <c r="C19" s="22"/>
       <c r="D19" s="19"/>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="U19" s="22"/>
     </row>
-    <row r="20" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="20" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B20" s="19"/>
       <c r="C20" s="20"/>
       <c r="D20" s="19"/>
@@ -5313,7 +5313,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="21" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B21" s="19"/>
       <c r="C21" s="21"/>
       <c r="D21" s="19"/>
@@ -5339,7 +5339,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="22" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B22" s="19"/>
       <c r="C22" s="22"/>
       <c r="D22" s="19"/>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="U22" s="22"/>
     </row>
-    <row r="23" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="23" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B23" s="19"/>
       <c r="C23" s="20"/>
       <c r="D23" s="19"/>
@@ -5389,7 +5389,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="24" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="24" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B24" s="19"/>
       <c r="C24" s="21"/>
       <c r="D24" s="19"/>
@@ -5415,7 +5415,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="25" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="25" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B25" s="19"/>
       <c r="C25" s="22"/>
       <c r="D25" s="19"/>
@@ -5441,7 +5441,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="26" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B26" s="19"/>
       <c r="C26" s="20"/>
       <c r="D26" s="19"/>
@@ -5467,7 +5467,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="27" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="27" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B27" s="19"/>
       <c r="C27" s="21"/>
       <c r="D27" s="19"/>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="U27" s="21"/>
     </row>
-    <row r="28" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="248.92" customHeight="true">
+    <row r="28" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="129.63" customHeight="true">
       <c r="B28" s="19"/>
       <c r="C28" s="22"/>
       <c r="D28" s="19"/>
@@ -5522,7 +5522,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="24"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="46"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>